<commit_message>
Fix real-data issues found on a 134k-row CSV
- Fast date parsing: shape checks, fromisoformat (timezone-aware ISO), caching
  (profiling 66 s -> 2.8 s on 134k rows)
- Re-validate corrected CSVs under the original sheet name; keep line endings
- Quality score is floored so it never shows 100% with errors present
- Identifier detection for hash-like ids; suggested length rule for them
- Profile flags dominant placeholder values in date/numeric columns
- UI checks the API URL is really IloveCSV; default port 8010; 25 MB limit
</commit_message>
<xml_diff>
--- a/reports/demo/demo_orders_audit.xlsx
+++ b/reports/demo/demo_orders_audit.xlsx
@@ -457,7 +457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>534a0830d353</t>
+          <t>a65149554b28</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ced905d3588631ef78d0173be18e1ba8d41a5e1e468fa903360ed4973fdcc3e0</t>
+          <t>9def0ed7ac687a655ebf5087e970e13744f54d0b5f5b6e58e9b5ee5b37d614d0</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>f3f73502006f9c7743632524ffde2c2fd6bcaf64575ac881d4f1698fb7b3b7f4</t>
+          <t>3d93520c4f5dd7c48be8cf3877f9a4d4596504cfab79375410757f4c5fdbc649</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3618,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-17T20:10:46+00:00</t>
+          <t>2026-10-18T04:22:36+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>

<commit_message>
Fix gaps found by an external noisy-workbook evaluation
- Duplicate records: compare rows ignoring a surrogate id (C001, C002...),
  case and spacing; natural keys such as hashes are still compared
- Suggested rules no longer legalise errors: numeric bounds from the
  non-outlier bulk, required when <=20% empty, Readme sheets skipped,
  full category lists
- New rule options: format email/phone (with fixes), aliases; built-in
  case-variant check with canonical-spelling fixes
- Quality score counts warnings (0.5) and whole duplicate rows; formula
  documented; rows reported per sheet
- Export with zero approvals is flagged in the UI, API and report; unsaved
  review decisions are saved on Next
- UI tables no longer crash on mixed-type columns
- Regression test reproducing the evaluation workbook
</commit_message>
<xml_diff>
--- a/reports/demo/demo_orders_audit.xlsx
+++ b/reports/demo/demo_orders_audit.xlsx
@@ -418,10 +418,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -457,7 +457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>a65149554b28</t>
+          <t>730e008c1085</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:19+00:00</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9def0ed7ac687a655ebf5087e970e13744f54d0b5f5b6e58e9b5ee5b37d614d0</t>
+          <t>8315871dd19de1c860e0b676491c19f094b9fb139b906772c4769da3e8224269</t>
         </is>
       </c>
     </row>
@@ -541,108 +541,150 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3d93520c4f5dd7c48be8cf3877f9a4d4596504cfab79375410757f4c5fdbc649</t>
+          <t>6ec37fe28dd861adc08bfc03c9bbb635ae2fabd17a71994e1e8b65bcde29cdfb</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rows checked</t>
+          <t>Rows checked: Orders</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>341</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Quality score (before)</t>
+          <t>Rows checked: Customers</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>99.48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Quality score (after)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>99.51000000000001</v>
+          <t>Quality score formula</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>100 x (1 - (cells with errors + 0.5 x cells with only warnings) / cells checked)</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Errors (before)</t>
+          <t>Quality score (before)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>99.09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Errors (after)</t>
+          <t>Quality score (after)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>99.22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Warnings (before)</t>
+          <t>Errors (before)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Warnings (after)</t>
+          <t>Errors (after)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Anomalies</t>
+          <t>Warnings (before)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Changes applied</t>
+          <t>Warnings (after)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Anomalies</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Changes applied</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Changes skipped</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B22" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Suggestions still pending (not applied)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Suggestions rejected</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2704,13 +2746,13 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>error</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Row repeats row 129 exactly.</t>
+          <t>Row repeats row 129 (ignoring order_id; case and spacing ignored).</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -3434,7 +3476,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3521,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3568,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3615,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3618,7 +3660,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3705,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3752,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3799,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3846,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3867,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -3904,7 +3946,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Row repeats row 129 exactly.</t>
+          <t>Row repeats row 129 (ignoring order_id; case and spacing ignored).</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -3925,7 +3967,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-18T04:22:36+00:00</t>
+          <t>2026-10-18T05:12:18+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>

<commit_message>
Make cleaning output honest: issue outcomes, unresolved marking, safe duplicates
- Every issue gets an outcome: resolved / open / pending_review / approved /
  rejected / dismissed; after export it is decided by re-validating the
  corrected file, with deleted rows mapped back to original row numbers
- Unresolved issues are listed (Unresolved sheet, report section, API filter)
  and highlighted with a comment in the corrected workbook; report says
  'Not fully clean' with counts
- Duplicates: configurable columns and match mode, a side-by-side preview
  (UI + /duplicates), and bulk approval never deletes rows unless asked
- Quality score shown with its numbers before and after
- Phones: numeric phone cells flagged and converted; digit strings written
  as Text-format cells
- Ambiguous dates resolved from unambiguous dates in the same column
- Report lists free-text columns whose spelling no rule verifies
- Forward-only DB migration for the new columns
</commit_message>
<xml_diff>
--- a/reports/demo/demo_orders_audit.xlsx
+++ b/reports/demo/demo_orders_audit.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Profile" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Issues" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Anomalies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Changes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Skipped" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Unresolved" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Profile" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Issues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Anomalies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Changes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Skipped" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -440,251 +441,309 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tool</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IloveCSV 0.1.0</t>
+          <t>NOT FULLY CLEAN: 18 error(s) and 0 warning(s) remain; see the Unresolved sheet</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Run id</t>
+          <t>Tool</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>730e008c1085</t>
+          <t>IloveCSV 0.1.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Validated at</t>
+          <t>Run id</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>05ee690e179f</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Exported at</t>
+          <t>Validated at</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:19+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Input file</t>
+          <t>Exported at</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>demo_orders.xlsx</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Input SHA-256</t>
+          <t>Input file</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>8315871dd19de1c860e0b676491c19f094b9fb139b906772c4769da3e8224269</t>
+          <t>demo_orders.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rules SHA-256</t>
+          <t>Input SHA-256</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1f44a51bf7cf6b2a3620a24fbfb93621b64c16548dd9146108ec2277281fc85d</t>
+          <t>146d95ec7a25a5a815efe3cfbcd4e4d7992640e67ed7615cddc97dfe3ac5de51</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Output file</t>
+          <t>Rules SHA-256</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>demo_orders_corrected.xlsx</t>
+          <t>1f44a51bf7cf6b2a3620a24fbfb93621b64c16548dd9146108ec2277281fc85d</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Output SHA-256</t>
+          <t>Output file</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6ec37fe28dd861adc08bfc03c9bbb635ae2fabd17a71994e1e8b65bcde29cdfb</t>
+          <t>demo_orders_corrected.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rows checked: Orders</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>301</v>
+          <t>Output SHA-256</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>d1eaa17344ad8f7eecc5922cb1ff96fc89778a6642c71f6a162aedd10f7ec0b0</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rows checked: Customers</t>
+          <t>Rows checked: Orders</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>40</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Quality score formula</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>100 x (1 - (cells with errors + 0.5 x cells with only warnings) / cells checked)</t>
-        </is>
+          <t>Rows checked: Customers</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Quality score (before)</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>99.09</v>
+          <t>Quality score formula</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>100 x (1 - (cells with errors + 0.5 x cells with only warnings) / cells checked)</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Quality score (after)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>99.22</v>
+          <t>Quality score (before)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>100 x (1 - (28 + 0.5 x 7) / 3471) = 99.09</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Errors (before)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>19</v>
+          <t>Quality score (after, from re-validating the corrected file)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>100 x (1 - (27 + 0.5 x 0) / 3471) = 99.22</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Errors (after)</t>
+          <t>Errors (before)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Warnings (before)</t>
+          <t>Errors unresolved (after)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Warnings (after)</t>
+          <t>Warnings (before)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Anomalies</t>
+          <t>Warnings unresolved (after)</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Changes applied</t>
+          <t>Anomalies</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Changes skipped</t>
+          <t>Issues resolved</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Suggestions still pending (not applied)</t>
+          <t>Issues open</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Issues pending_review</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Changes applied</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Changes skipped</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Suggestions still pending (not applied)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Suggestions rejected</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>0</v>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Spelling not verified (no reference list)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Orders.channel</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -693,6 +752,862 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>corrected_cell_ref</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>original_cell_ref</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rule_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resolution</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>resolution_note</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>introduced_by_fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Orders!A38</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Orders!A38</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>'order_id' is required but empty.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Orders!A156</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Orders!A156</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ORD-12A4</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>'ORD-12A4' does not match the pattern ^ORD-\d{5}$.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Orders!B20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Orders!B20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>not a date</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>'not a date' is not a date.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Orders!B62</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Orders!B62</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>range</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2019-05-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2019-05-01 is below the minimum 2020-01-01.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Orders!B260</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Orders!B260</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>not_future</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2031-01-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2031-01-01 is in the future.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Orders!D291</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Orders!D291</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>'customer_id' is required but empty.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orders!E131</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Orders!E131</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>allowed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Lost</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>'Lost' is not an allowed value for 'status'.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Orders!G121</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Orders!G121</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>'abc' is not a number.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Orders!G59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Orders!G59</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>range</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5000 is above the maximum 1000.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Orders!G92</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Orders!G92</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>range</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0 is below the minimum 1.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Orders!K16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Orders!K16</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>regex</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>not-an-email</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>'not-an-email' does not match the pattern ^[\w.+-]+@[\w-]+\.[\w.]+$.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Orders!A302</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Orders!A302</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>key.duplicate</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ORD-00128</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Duplicate key (ORD-00128); first seen in row 129.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Orders!A302</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Orders!A302</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>row.duplicate</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Row repeats row 129 (ignoring order_id; case and spacing ignored).</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Approved fix not effective: workbook contains formulas; deleting rows could break references, so the row was kept and marked.</t>
+        </is>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Orders!C278</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Orders!C278</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ship_after_order</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2024-09-21T00:00:00</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ship date is before the order date (ship_date=2024-09-21, order_date=2024-09-24)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Orders!J135</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Orders!J135</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>total_matches</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>19848.4</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Total does not equal quantity x unit price (total=19848.4, quantity=30, unit_price=658.28)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>pending_review</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Suggested fix (rule_fix) was not reviewed.</t>
+        </is>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Orders!C75</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Orders!C75</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>shipped_needs_date</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>'ship_date' is required when status == 'Shipped'.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Appeared after corrections were applied (for example, a corrected category now triggers another rule).</t>
+        </is>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Orders!C282</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Orders!C282</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>shipped_needs_date</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>'ship_date' is required when status == 'Shipped'.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Orders!D22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Orders!D22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>customer_exists</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>C999</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>'C999' was not found in Customers.customer_id.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1675,13 +2590,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1692,8 +2607,9 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1739,12 +2655,17 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>resolution</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>resolution_note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>why</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>status</t>
         </is>
       </c>
     </row>
@@ -1787,12 +2708,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>A required field is empty, so downstream reports and joins will miss this record.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -1839,12 +2765,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>The value does not follow the required format.</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -1891,12 +2822,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>The value cannot be read as the expected type, so calculations or sorting on this column will fail or skip it.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -1943,12 +2879,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Fixed by text_to_date; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>The date is stored as text, so date filters, sorting and arithmetic will treat it as a string.</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -1993,12 +2934,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fixed by serial_to_date; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>An Excel serial number sits where a date is expected; it is probably a date whose formatting was lost.</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2045,12 +2991,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>The value is outside the range the rules allow, which usually means a typo or a unit mistake.</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2097,12 +3048,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>The date lies in the future, which is impossible for this field.</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2145,12 +3101,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>A required field is empty, so downstream reports and joins will miss this record.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2197,12 +3158,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Fixed by canonical_category; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>The category is valid but spelled with different case or spacing, which splits one group into several.</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2249,12 +3215,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Fixed by fuzzy_category; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>The value is not in the list of allowed categories, so it will be miscounted in any grouping.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2301,12 +3272,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>The value is not in the list of allowed categories, so it will be miscounted in any grouping.</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2353,12 +3329,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Fixed by text_to_number; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>The value is a number or boolean stored as text; Excel and most tools will not sum or compare it correctly.</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2405,12 +3386,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
           <t>The value cannot be read as the expected type, so calculations or sorting on this column will fail or skip it.</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2455,12 +3441,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t>The value is outside the range the rules allow, which usually means a typo or a unit mistake.</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2505,12 +3496,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>The value is outside the range the rules allow, which usually means a typo or a unit mistake.</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2557,12 +3553,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Fixed by text_to_number; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
           <t>The value is a number or boolean stored as text; Excel and most tools will not sum or compare it correctly.</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2609,12 +3610,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>The value does not follow the required format.</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2661,12 +3667,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
           <t>Two rows share the same key, so lookups on this key are ambiguous.</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2713,12 +3724,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Fixed by trim_whitespace; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>Leading, trailing or repeated spaces make equal values look different to filters and lookups.</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2757,12 +3773,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Approved fix not effective: workbook contains formulas; deleting rows could break references, so the row was kept and marked.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>The whole row repeats an earlier row; totals that include both will double-count.</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2809,12 +3830,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t>A cross-column business rule from the rule file was not satisfied.</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2859,12 +3885,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>pending_review</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Suggested fix (rule_fix) was not reviewed.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
           <t>A cross-column business rule from the rule file was not satisfied.</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2907,12 +3938,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>A cross-column business rule from the rule file was not satisfied.</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -2959,12 +3995,17 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>No safe automatic correction exists; fix the source data by hand.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>A cross-column business rule from the rule file was not satisfied.</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -3011,12 +4052,17 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Fixed by fuzzy_category; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t>The value is not in the list of allowed categories, so it will be miscounted in any grouping.</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -3063,12 +4109,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Fixed by canonical_category; passes re-validation.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
           <t>The category is valid but spelled with different case or spacing, which splits one group into several.</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>open</t>
         </is>
       </c>
     </row>
@@ -3077,13 +4128,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3095,6 +4146,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3143,6 +4195,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>resolution</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3186,6 +4243,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>pending_review</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3229,6 +4291,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>pending_review</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3274,6 +4341,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>pending_review</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3317,6 +4389,11 @@
           <t>open</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>pending_review</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3358,6 +4435,11 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>open</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>pending_review</t>
         </is>
       </c>
     </row>
@@ -3366,7 +4448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3476,7 +4558,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3521,7 +4603,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3568,7 +4650,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3615,7 +4697,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3660,7 +4742,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3705,7 +4787,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3752,7 +4834,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3799,7 +4881,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3846,7 +4928,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
     </row>
@@ -3855,7 +4937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3967,7 +5049,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:12:18+00:00</t>
+          <t>2026-10-18T05:52:56+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>